<commit_message>
Added new parts and their mass to parts_list + added new models for components
</commit_message>
<xml_diff>
--- a/design/parts_list.xlsx
+++ b/design/parts_list.xlsx
@@ -8,24 +8,35 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Desktop\BOB\BOB\design\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5696305A-EA9B-4ED7-A170-C96A0B6401EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0DB88467-114D-4779-B4CE-C5EA834449BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10560" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="18">
   <si>
     <t>Parts</t>
   </si>
@@ -45,13 +56,40 @@
     <t>Given</t>
   </si>
   <si>
-    <t>6?</t>
-  </si>
-  <si>
     <t xml:space="preserve">HC-SR04 Ultrasonic Sensor </t>
   </si>
   <si>
     <t>N.A.</t>
+  </si>
+  <si>
+    <t>Total Mass</t>
+  </si>
+  <si>
+    <t>Battery</t>
+  </si>
+  <si>
+    <t>Mass (g)</t>
+  </si>
+  <si>
+    <t>Motor driver L298N</t>
+  </si>
+  <si>
+    <t>N20 DC GEARED MOTOR</t>
+  </si>
+  <si>
+    <t>Sum</t>
+  </si>
+  <si>
+    <t>Wheels???</t>
+  </si>
+  <si>
+    <t>TCRT5000 Infrared Tracking Sensor Module</t>
+  </si>
+  <si>
+    <t>Remainder</t>
+  </si>
+  <si>
+    <t>Rollers</t>
   </si>
 </sst>
 </file>
@@ -378,13 +416,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:G11"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="38" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -397,8 +435,14 @@
       <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -406,24 +450,164 @@
         <v>1</v>
       </c>
       <c r="C2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D2" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E2">
+        <v>25</v>
+      </c>
+      <c r="F2">
+        <f>B2*E2</f>
+        <v>25</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3">
+        <v>6</v>
+      </c>
+      <c r="C3" t="s">
         <v>7</v>
-      </c>
-      <c r="B3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C3" t="s">
-        <v>8</v>
       </c>
       <c r="D3" t="s">
         <v>5</v>
+      </c>
+      <c r="E3">
+        <v>9</v>
+      </c>
+      <c r="F3">
+        <f t="shared" ref="F3:F9" si="0">B3*E3</f>
+        <v>54</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4">
+        <v>1</v>
+      </c>
+      <c r="C4" t="s">
+        <v>7</v>
+      </c>
+      <c r="D4" t="s">
+        <v>5</v>
+      </c>
+      <c r="E4">
+        <v>200</v>
+      </c>
+      <c r="F4">
+        <f t="shared" si="0"/>
+        <v>200</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>11</v>
+      </c>
+      <c r="B5">
+        <v>1</v>
+      </c>
+      <c r="C5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D5" t="s">
+        <v>5</v>
+      </c>
+      <c r="E5">
+        <v>33</v>
+      </c>
+      <c r="F5">
+        <f t="shared" si="0"/>
+        <v>33</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B6">
+        <v>2</v>
+      </c>
+      <c r="C6" t="s">
+        <v>7</v>
+      </c>
+      <c r="D6" t="s">
+        <v>5</v>
+      </c>
+      <c r="E6">
+        <v>10</v>
+      </c>
+      <c r="F6">
+        <f t="shared" si="0"/>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>14</v>
+      </c>
+      <c r="B7">
+        <v>2</v>
+      </c>
+      <c r="F7">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>15</v>
+      </c>
+      <c r="B8">
+        <v>2</v>
+      </c>
+      <c r="C8" t="s">
+        <v>7</v>
+      </c>
+      <c r="D8" t="s">
+        <v>5</v>
+      </c>
+      <c r="E8">
+        <v>17</v>
+      </c>
+      <c r="F8">
+        <f t="shared" si="0"/>
+        <v>34</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>17</v>
+      </c>
+      <c r="B9">
+        <v>2</v>
+      </c>
+      <c r="F9">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="F10" s="1">
+        <f>SUM(F2:F8)</f>
+        <v>366</v>
+      </c>
+      <c r="G10" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="F11">
+        <f>500-F10</f>
+        <v>134</v>
+      </c>
+      <c r="G11" s="1" t="s">
+        <v>16</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated parts list, components, shell and assembly
</commit_message>
<xml_diff>
--- a/design/parts_list.xlsx
+++ b/design/parts_list.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="26827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="26924"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Desktop\BOB\BOB\design\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0DB88467-114D-4779-B4CE-C5EA834449BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2131742F-70BE-43F4-9793-0940140B3CD1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10560" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="18">
   <si>
     <t>Parts</t>
   </si>
@@ -50,9 +50,6 @@
     <t>Cost</t>
   </si>
   <si>
-    <t>Arduino UNO</t>
-  </si>
-  <si>
     <t>Given</t>
   </si>
   <si>
@@ -80,16 +77,19 @@
     <t>Sum</t>
   </si>
   <si>
-    <t>Wheels???</t>
-  </si>
-  <si>
-    <t>TCRT5000 Infrared Tracking Sensor Module</t>
-  </si>
-  <si>
     <t>Remainder</t>
   </si>
   <si>
     <t>Rollers</t>
+  </si>
+  <si>
+    <t>43MM N20</t>
+  </si>
+  <si>
+    <t>Hailege ESP32 ESP-32S ESP-WROOM-32</t>
+  </si>
+  <si>
+    <t>qrt-1a Infrared</t>
   </si>
 </sst>
 </file>
@@ -436,66 +436,66 @@
         <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="B2">
         <v>1</v>
       </c>
       <c r="C2" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D2" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E2">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="F2">
         <f>B2*E2</f>
-        <v>25</v>
+        <v>10</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B3">
+        <v>4</v>
+      </c>
+      <c r="C3" t="s">
         <v>6</v>
       </c>
-      <c r="B3">
-        <v>6</v>
-      </c>
-      <c r="C3" t="s">
-        <v>7</v>
-      </c>
       <c r="D3" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E3">
         <v>9</v>
       </c>
       <c r="F3">
         <f t="shared" ref="F3:F9" si="0">B3*E3</f>
-        <v>54</v>
+        <v>36</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B4">
         <v>1</v>
       </c>
       <c r="C4" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D4" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E4">
         <v>200</v>
@@ -507,16 +507,16 @@
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B5">
         <v>1</v>
       </c>
       <c r="C5" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D5" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E5">
         <v>33</v>
@@ -528,16 +528,16 @@
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B6">
         <v>2</v>
       </c>
       <c r="C6" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E6">
         <v>10</v>
@@ -549,28 +549,37 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B7">
         <v>2</v>
       </c>
+      <c r="C7" t="s">
+        <v>6</v>
+      </c>
+      <c r="D7" t="s">
+        <v>4</v>
+      </c>
+      <c r="E7">
+        <v>19</v>
+      </c>
       <c r="F7">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>38</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B8">
         <v>2</v>
       </c>
       <c r="C8" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D8" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E8">
         <v>17</v>
@@ -582,7 +591,7 @@
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="B9">
         <v>2</v>
@@ -595,19 +604,19 @@
     <row r="10" spans="1:7" x14ac:dyDescent="0.35">
       <c r="F10" s="1">
         <f>SUM(F2:F8)</f>
-        <v>366</v>
+        <v>371</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.35">
       <c r="F11">
         <f>500-F10</f>
-        <v>134</v>
+        <v>129</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Version 2 of BOB Model
</commit_message>
<xml_diff>
--- a/design/parts_list.xlsx
+++ b/design/parts_list.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="26924"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27231"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Desktop\BOB\BOB\design\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Desktop\BOB\design\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2131742F-70BE-43F4-9793-0940140B3CD1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F1747E9-2FE6-491C-A4B1-12A0DAEA3B6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10560" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="17">
   <si>
     <t>Parts</t>
   </si>
@@ -78,9 +78,6 @@
   </si>
   <si>
     <t>Remainder</t>
-  </si>
-  <si>
-    <t>Rollers</t>
   </si>
   <si>
     <t>43MM N20</t>
@@ -444,7 +441,7 @@
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B2">
         <v>1</v>
@@ -468,7 +465,7 @@
         <v>5</v>
       </c>
       <c r="B3">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C3" t="s">
         <v>6</v>
@@ -481,7 +478,7 @@
       </c>
       <c r="F3">
         <f t="shared" ref="F3:F9" si="0">B3*E3</f>
-        <v>36</v>
+        <v>18</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.35">
@@ -549,7 +546,7 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B7">
         <v>2</v>
@@ -570,7 +567,7 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B8">
         <v>2</v>
@@ -589,22 +586,10 @@
         <v>34</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A9" t="s">
-        <v>14</v>
-      </c>
-      <c r="B9">
-        <v>2</v>
-      </c>
-      <c r="F9">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.35">
       <c r="F10" s="1">
         <f>SUM(F2:F8)</f>
-        <v>371</v>
+        <v>353</v>
       </c>
       <c r="G10" s="1" t="s">
         <v>12</v>
@@ -613,7 +598,7 @@
     <row r="11" spans="1:7" x14ac:dyDescent="0.35">
       <c r="F11">
         <f>500-F10</f>
-        <v>129</v>
+        <v>147</v>
       </c>
       <c r="G11" s="1" t="s">
         <v>13</v>

</xml_diff>

<commit_message>
Final model revision before print
</commit_message>
<xml_diff>
--- a/design/parts_list.xlsx
+++ b/design/parts_list.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Desktop\BOB\design\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9F486F8-C927-4589-B6D5-87BE3CF08A5A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8718F6C7-18EA-408A-8EA3-9B1BF5AB31D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10560" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="19">
   <si>
     <t>Parts</t>
   </si>
@@ -87,6 +87,12 @@
   </si>
   <si>
     <t>QTR-1A Infrared</t>
+  </si>
+  <si>
+    <t>Mass of Shell</t>
+  </si>
+  <si>
+    <t>Estimated</t>
   </si>
 </sst>
 </file>
@@ -586,10 +592,31 @@
         <v>0.4</v>
       </c>
     </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>17</v>
+      </c>
+      <c r="B9">
+        <v>1</v>
+      </c>
+      <c r="C9" t="s">
+        <v>6</v>
+      </c>
+      <c r="D9" t="s">
+        <v>18</v>
+      </c>
+      <c r="E9">
+        <v>139.03</v>
+      </c>
+      <c r="F9">
+        <f>B9*E9</f>
+        <v>139.03</v>
+      </c>
+    </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.35">
       <c r="F10" s="1">
-        <f>SUM(F2:F8)</f>
-        <v>319.39999999999998</v>
+        <f>SUM(F2:F9)</f>
+        <v>458.42999999999995</v>
       </c>
       <c r="G10" s="1" t="s">
         <v>12</v>
@@ -598,7 +625,7 @@
     <row r="11" spans="1:7" x14ac:dyDescent="0.35">
       <c r="F11">
         <f>500-F10</f>
-        <v>180.60000000000002</v>
+        <v>41.57000000000005</v>
       </c>
       <c r="G11" s="1" t="s">
         <v>13</v>

</xml_diff>